<commit_message>
Regenerate the instance sheet blank
Test runs had left a stray =SUM() and a check column in the shipped
example. Rebuilt from make_instance.py so it opens with names only.
</commit_message>
<xml_diff>
--- a/实例成绩表.xlsx
+++ b/实例成绩表.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,27 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font/>
-    <font>
-      <color rgb="FF006100"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF9C0006"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFFC7CE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,11 +46,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,328 +418,202 @@
   </sheetPr>
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>姓名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>第一题</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>第二题</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>第三题</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>第四题</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>总分</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>核对</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>王小明</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F2">
-        <f>SUM(B2:E2)</f>
-        <v/>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>李四</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>18</v>
-      </c>
-      <c r="E3" t="n">
-        <v>70</v>
-      </c>
-      <c r="F3">
-        <f>SUM(B3:E3)</f>
-        <v/>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>不一致</t>
-        </is>
-      </c>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>张伟</t>
         </is>
       </c>
-      <c r="F4">
-        <f>SUM(B4:E4)</f>
-        <v/>
-      </c>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
       <c r="G4" s="1" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>刘洋</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>12</v>
-      </c>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="n">
-        <v>12</v>
-      </c>
-      <c r="E5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F5">
-        <f>SUM(B5:E5)</f>
-        <v/>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="B5" s="1" t="n"/>
+      <c r="C5" s="1" t="n"/>
+      <c r="D5" s="1" t="n"/>
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>陈静</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <f>SUM(B6:E6)</f>
-        <v/>
-      </c>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
       <c r="G6" s="1" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>张三</t>
         </is>
       </c>
-      <c r="F7">
-        <f>SUM(B7:E7)</f>
-        <v/>
-      </c>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="1" t="n"/>
       <c r="G7" s="1" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>赵磊</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C8" t="n">
-        <v>12</v>
-      </c>
-      <c r="D8" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" t="n">
-        <v>10</v>
-      </c>
-      <c r="F8">
-        <f>SUM(B8:E8)</f>
-        <v/>
-      </c>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
       <c r="G8" s="1" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>孙丽</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E9" t="n">
-        <v>8</v>
-      </c>
-      <c r="F9">
-        <f>SUM(B9:E9)</f>
-        <v/>
-      </c>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="n"/>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
       <c r="G9" s="1" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>周杰</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>7</v>
-      </c>
-      <c r="C10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10">
-        <f>SUM(B10:E10)</f>
-        <v/>
-      </c>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
       <c r="G10" s="1" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>吴敏</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>12</v>
-      </c>
-      <c r="C11" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" t="n">
-        <v>90</v>
-      </c>
-      <c r="E11" t="n">
-        <v>77</v>
-      </c>
-      <c r="F11">
-        <f>SUM(B11:E11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>不一致</t>
-        </is>
-      </c>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>郑浩</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" t="n">
-        <v>15</v>
-      </c>
-      <c r="E12" t="n">
-        <v>18</v>
-      </c>
-      <c r="F12">
-        <f>SUM(B12:E12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>张三</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13">
-        <f>SUM(B13:E13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
+      <c r="D13" s="1" t="n"/>
+      <c r="E13" s="1" t="n"/>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>